<commit_message>
feat: Standardize payment method display names for improved output formatting
</commit_message>
<xml_diff>
--- a/output/BBVA_VISA_20250430.xlsx
+++ b/output/BBVA_VISA_20250430.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>

</xml_diff>